<commit_message>
Hide small-sample search indices and explain low-baseline limits
</commit_message>
<xml_diff>
--- a/user_summary_review/字段计算公式说明.xlsx
+++ b/user_summary_review/字段计算公式说明.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'重点词看板25列'!$A$1:$F$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'总表71列'!$A$1:$F$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'使用说明'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'使用说明'!$A$1:$B$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -908,22 +908,22 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>指数计算</t>
+          <t>有展示筛选的指数</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>样本CTR÷市场CTR</t>
+          <t>样本CTR÷市场CTR；样本点击&lt;100时留空</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>=IFERROR(IF(AND(ISNUMBER(H2),ISNUMBER(I2),I2&gt;0),H2/I2,""),"")</t>
+          <t>=IFERROR(IF(AND(ISNUMBER(E2),E2&gt;=100,ISNUMBER(H2),ISNUMBER(I2),I2&gt;0),H2/I2,""),"")</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>普通小数或倍数，1倍为描述性基准。</t>
+          <t>倍数仅辅助描述；100点击是展示筛选线，不保证稳定。低市场CTR会放大倍数，须看曝光、点击和绝对率。</t>
         </is>
       </c>
     </row>
@@ -940,22 +940,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>指数计算</t>
+          <t>有展示筛选的指数</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>样本点击后购买比÷市场点击后购买比</t>
+          <t>样本点击后购买比÷市场点击后购买比；样本点击&lt;100时留空</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>=IFERROR(IF(AND(ISNUMBER(L2),ISNUMBER(M2),M2&gt;0),L2/M2,""),"")</t>
+          <t>=IFERROR(IF(AND(ISNUMBER(E2),E2&gt;=100,ISNUMBER(L2),ISNUMBER(M2),M2&gt;0),L2/M2,""),"")</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>不是显著性检验。</t>
+          <t>不是显著性检验；仍须核查购买计数和绝对率，不能按倍数排名。</t>
         </is>
       </c>
     </row>
@@ -2843,22 +2843,22 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>比率或指数计算</t>
+          <t>有展示筛选的指数</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>样本曝光CTR÷市场曝光CTR</t>
+          <t>样本曝光CTR÷市场曝光CTR；样本点击&lt;100时留空</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>=IFERROR(IF(AND(ISNUMBER(N2),ISNUMBER(L2),L2&gt;0),N2/L2,""),"")</t>
+          <t>=IFERROR(IF(AND(ISNUMBER(M2),M2&gt;=100,ISNUMBER(N2),ISNUMBER(L2),L2&gt;0),N2/L2,""),"")</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>任一输入非数字、分母0或缺失均留空；不要额外乘100，百分比由单元格格式显示。</t>
+          <t>普通小数/倍数；100点击是展示筛选线，不是显著性或稳定性保证。低市场基准放大比值，先看原始计数和绝对率，不按指数大小排序。</t>
         </is>
       </c>
     </row>
@@ -2875,22 +2875,22 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>比率或指数计算</t>
+          <t>有展示筛选的指数</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>样本点击后购买比÷市场点击后购买比</t>
+          <t>样本点击后购买比÷市场点击后购买比；样本点击&lt;100时留空</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>=IFERROR(IF(AND(ISNUMBER(AP2),ISNUMBER(AK2),AK2&gt;0),AP2/AK2,""),"")</t>
+          <t>=IFERROR(IF(AND(ISNUMBER(M2),M2&gt;=100,ISNUMBER(AP2),ISNUMBER(AK2),AK2&gt;0),AP2/AK2,""),"")</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>任一输入非数字、分母0或缺失均留空；不要额外乘100，百分比由单元格格式显示。</t>
+          <t>普通小数/倍数；100点击是展示筛选线，不是显著性或稳定性保证。低市场基准放大比值，先看原始计数和绝对率，不按指数大小排序。</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3656,65 +3656,77 @@
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>市场去重</t>
+          <t>指数展示筛选</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>同词市场搜索、曝光、点击、加购、购买值一致后只取一次；ASIN计数可按已收录ASIN求和。</t>
+          <t>看板N/O与总表AW/AX仅在样本点击≥100且上游有效时显示。少于100时保留计数与绝对率，指数留空；100不是统计显著性门槛。市场基准极低仍须核查，不用倍数排名。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>价格和排名</t>
+          <t>市场去重</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>市场/ASIN中位数取原始值；跨ASIN整体中位数无法精确还原，不计算。ASIN排名不平均成品牌排名。</t>
+          <t>同词市场搜索、曝光、点击、加购、购买值一致后只取一次；ASIN计数可按已收录ASIN求和。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>自然量</t>
+          <t>价格和排名</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>理论上同范围完整总量减广告量可分解；本次范围与购买归因未对齐，不计算自然量、广告占比。</t>
+          <t>市场/ASIN中位数取原始值；跨ASIN整体中位数无法精确还原，不计算。ASIN排名不平均成品牌排名。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="72" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>覆盖与版本</t>
+          <t>自然量</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2410个词只覆盖部分广告，范围固定在当前输入版本。新增原始数据时应更新公式范围，并重新核对计数和结论。</t>
+          <t>理论上同范围完整总量减广告量可分解；本次范围与购买归因未对齐，不计算自然量、广告占比。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="72" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>覆盖与版本</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2410个词只覆盖部分广告，范围固定在当前输入版本。新增原始数据时应更新公式范围，并重新核对计数和结论。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>兼容性</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>XLOOKUP、FILTER和UNIQUE需要支持这些函数的Excel/WPS版本。指南是公式说明，不会修改主数据工作簿。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B15"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>